<commit_message>
se ajust 1-reglas sobre los turnos para que no 3 turnos dia ni 3 turnos noches 2-tablero de inicio con notificaciones de novedades.
</commit_message>
<xml_diff>
--- a/sgturnos/mallas/malla_med03_2026-01.xlsx
+++ b/sgturnos/mallas/malla_med03_2026-01.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="47">
   <si>
     <t>Empleado</t>
   </si>
@@ -125,15 +125,15 @@
     <t>CP3h+AP9h</t>
   </si>
   <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
     <t>LB</t>
   </si>
   <si>
-    <t>TN</t>
-  </si>
-  <si>
-    <t>PT</t>
-  </si>
-  <si>
     <t>16</t>
   </si>
   <si>
@@ -153,9 +153,6 @@
   </si>
   <si>
     <t>Carlos Rodríguez</t>
-  </si>
-  <si>
-    <t>AP12h</t>
   </si>
 </sst>
 </file>
@@ -386,89 +383,89 @@
       <c r="D2" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="E2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="F2" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="G2" t="s" s="5">
+      <c r="E2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="F2" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s" s="4">
         <v>39</v>
       </c>
       <c r="H2" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="I2" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="J2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="K2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="L2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="M2" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="N2" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="O2" t="s" s="1">
-        <v>35</v>
+      <c r="I2" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="J2" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="K2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="M2" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="N2" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="O2" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="P2" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="Q2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="R2" t="s" s="4">
-        <v>37</v>
+      <c r="Q2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="S2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="T2" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="U2" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="T2" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="U2" t="s" s="4">
         <v>39</v>
       </c>
       <c r="V2" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="W2" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="X2" t="s" s="4">
-        <v>37</v>
+      <c r="W2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="X2" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="Y2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="Z2" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AA2" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AB2" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AC2" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="AD2" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AE2" t="s" s="1">
-        <v>35</v>
+        <v>39</v>
+      </c>
+      <c r="Z2" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AA2" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AB2" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AC2" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AD2" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="AE2" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="AF2" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="AG2" t="s" s="0">
         <v>40</v>
@@ -491,88 +488,88 @@
         <v>35</v>
       </c>
       <c r="E3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="F3" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="G3" t="s" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="I3" t="s" s="1">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="I3" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="J3" t="s" s="1">
         <v>35</v>
       </c>
       <c r="K3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="L3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="M3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="N3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="O3" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="L3" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="M3" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="O3" t="s" s="4">
         <v>39</v>
       </c>
       <c r="P3" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="Q3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="R3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="S3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="T3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="U3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="V3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="W3" t="s" s="5">
+      <c r="Q3" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="R3" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="S3" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="T3" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="U3" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="V3" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="W3" t="s" s="4">
         <v>39</v>
       </c>
       <c r="X3" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="Y3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="Z3" t="s" s="4">
-        <v>37</v>
+      <c r="Y3" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="Z3" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="AA3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AB3" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AC3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AD3" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="AE3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AF3" t="s" s="1">
-        <v>35</v>
+        <v>39</v>
+      </c>
+      <c r="AB3" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AC3" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AD3" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AE3" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AF3" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="AG3" t="s" s="0">
         <v>40</v>
@@ -586,97 +583,97 @@
         <v>43</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="E4" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s" s="1">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="D4" t="s" s="6">
+        <v>36</v>
+      </c>
+      <c r="E4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="G4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="H4" t="s" s="6">
-        <v>36</v>
-      </c>
-      <c r="I4" t="s" s="4">
-        <v>37</v>
+      <c r="H4" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="J4" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="K4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="L4" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="K4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="L4" t="s" s="4">
         <v>39</v>
       </c>
       <c r="M4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="N4" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="O4" t="s" s="4">
-        <v>37</v>
+      <c r="N4" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="O4" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="P4" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="R4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="S4" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="T4" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="U4" t="s" s="1">
-        <v>35</v>
+      <c r="R4" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="S4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="T4" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="U4" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="V4" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="W4" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="W4" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="X4" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="Y4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="Z4" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="AA4" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AB4" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AC4" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="Y4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="Z4" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AA4" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="AB4" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AC4" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="AD4" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AE4" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AF4" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="AE4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AF4" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="AG4" t="s" s="0">
         <v>40</v>
@@ -695,92 +692,92 @@
       <c r="C5" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="D5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="E5" t="s" s="1">
-        <v>35</v>
+      <c r="D5" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="E5" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="F5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="H5" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="I5" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="K5" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="L5" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="M5" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="G5" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="I5" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="L5" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="M5" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="N5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="O5" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="O5" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="P5" t="s" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="Q5" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="R5" t="s" s="1">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="R5" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="S5" t="s" s="1">
         <v>35</v>
       </c>
       <c r="T5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="U5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="V5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="W5" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="X5" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="U5" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="V5" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="W5" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="X5" t="s" s="4">
         <v>39</v>
       </c>
       <c r="Y5" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="Z5" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AA5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AB5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AC5" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AD5" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AE5" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="AF5" t="s" s="1">
-        <v>35</v>
+      <c r="Z5" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AA5" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AB5" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AC5" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="AD5" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AE5" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AF5" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="AG5" t="s" s="0">
         <v>40</v>
@@ -800,90 +797,90 @@
         <v>35</v>
       </c>
       <c r="D6" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="F6" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="G6" t="s" s="4">
-        <v>37</v>
+      <c r="F6" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="H6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="I6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="J6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="K6" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="L6" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="M6" t="s" s="1">
-        <v>35</v>
+        <v>39</v>
+      </c>
+      <c r="I6" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="J6" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="K6" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="L6" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="M6" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="N6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="O6" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="O6" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="P6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="Q6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="R6" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="S6" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="T6" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="U6" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R6" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="S6" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="T6" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="U6" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="V6" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W6" t="s" s="1">
         <v>35</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="Y6" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="Z6" t="s" s="1">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="Z6" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="AA6" t="s" s="1">
         <v>35</v>
       </c>
       <c r="AB6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AC6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AD6" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AE6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AF6" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="AC6" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AD6" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AE6" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="AF6" t="s" s="4">
         <v>39</v>
       </c>
       <c r="AG6" t="s" s="0">
@@ -901,94 +898,94 @@
         <v>36</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="F7" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="G7" t="s" s="1">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="E7" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="G7" t="s" s="4">
+        <v>39</v>
       </c>
       <c r="H7" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="I7" t="s" s="3">
-        <v>47</v>
-      </c>
-      <c r="J7" t="s" s="3">
-        <v>47</v>
+      <c r="I7" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="J7" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="K7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="L7" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="M7" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="L7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="M7" t="s" s="4">
         <v>39</v>
       </c>
       <c r="N7" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="O7" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="P7" t="s" s="4">
-        <v>37</v>
+      <c r="O7" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="P7" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="Q7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="R7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="S7" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="T7" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="U7" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="V7" t="s" s="1">
-        <v>35</v>
+        <v>39</v>
+      </c>
+      <c r="R7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="S7" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="T7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="U7" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="V7" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="W7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="X7" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="X7" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="Y7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="Z7" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AA7" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="AB7" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AC7" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AD7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AE7" t="s" s="4">
-        <v>37</v>
-      </c>
-      <c r="AF7" t="s" s="4">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="Z7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AA7" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AB7" t="s" s="5">
+        <v>38</v>
+      </c>
+      <c r="AC7" t="s" s="4">
+        <v>39</v>
+      </c>
+      <c r="AD7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="AE7" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="AF7" t="s" s="5">
+        <v>38</v>
       </c>
       <c r="AG7" t="s" s="0">
         <v>40</v>

</xml_diff>